<commit_message>
chore: add new air quality CSV datasets and transformation documentation screenshot
</commit_message>
<xml_diff>
--- a/data/SetPointLimit.xlsx
+++ b/data/SetPointLimit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ex_work\AirQualityReview_Project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C6D2BAA-06F9-49AD-A50F-453276849561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D663E787-B07D-449B-8242-613508679203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7200" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2113,7 +2113,7 @@
         <v>479</v>
       </c>
       <c r="G2" s="4">
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="H2" s="3">
         <v>10</v>

</xml_diff>